<commit_message>
TP2-3: Implementar análisis de ventas
</commit_message>
<xml_diff>
--- a/datos/dataset.xlsx
+++ b/datos/dataset.xlsx
@@ -23,9 +23,41 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="9">
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Precio</t>
+  </si>
+  <si>
+    <t>Gaseosa</t>
+  </si>
+  <si>
+    <t>Alfajor</t>
+  </si>
+  <si>
+    <t>Papas Fritas</t>
+  </si>
+  <si>
+    <t>Chocolate</t>
+  </si>
+  <si>
+    <t>Caramelos</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -33,16 +65,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,12 +102,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -336,9 +412,240 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="16.05078125" customWidth="1"/>
+    <col min="2" max="2" width="17.68359375" customWidth="1"/>
+    <col min="3" max="3" width="13.578125" customWidth="1"/>
+    <col min="4" max="4" width="16.9453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="2">
+        <v>45662</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="2">
+        <v>45662</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="2">
+        <v>45665</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="2">
+        <v>45669</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="3">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="2">
+        <v>45672</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="2">
+        <v>45677</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="2">
+        <v>45691</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3">
+        <v>6</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="2">
+        <v>45695</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="2">
+        <v>45698</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3">
+        <v>4</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="2">
+        <v>45706</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="2">
+        <v>45717</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="2">
+        <v>45721</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="3">
+        <v>15</v>
+      </c>
+      <c r="D13" s="3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="2">
+        <v>45728</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="3">
+        <v>5</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="2">
+        <v>45736</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="3">
+        <v>6</v>
+      </c>
+      <c r="D15" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="2">
+        <v>45741</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1800</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>